<commit_message>
analyzing campagin2 test data
</commit_message>
<xml_diff>
--- a/src/tools/xil-data-analysis/2021-Toyota-Rav4-Prime/output-file/auxiliary-analysis-hv-with-pid.xlsx
+++ b/src/tools/xil-data-analysis/2021-Toyota-Rav4-Prime/output-file/auxiliary-analysis-hv-with-pid.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ddas\Documents\deb-anl-xil\src\tools\xil-data-analysis\2021-Toyota-Rav4-Prime\output-file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A40A61-4368-463B-B07D-8721078A7473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE76BFB-25B5-4CCD-B00E-3A98B5B9DA34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -912,7 +912,7 @@
         <v>0.25</v>
       </c>
       <c r="D2">
-        <v>79.799999999999031</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>